<commit_message>
Resolve multi-vehicle telemetry loop, mode clashing, and CORS blocks for parameter metadata
</commit_message>
<xml_diff>
--- a/test_frontend/reports/integration_test_report.xlsx
+++ b/test_frontend/reports/integration_test_report.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>34cf857</t>
+          <t>054419c</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-18 13:51:38</t>
+          <t>2026-06-19 11:29:24</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>1.01 s</t>
+          <t>1.05 s</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>4.73 s</t>
+          <t>4.82 s</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>0.33 s</t>
+          <t>0.24 s</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="E3" s="6" t="n">
-        <v>147</v>
+        <v>454</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>71</v>
+        <v>120</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>5702</v>
+        <v>5891</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>4800</v>
+        <v>4950</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>51</v>
+        <v>99</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>1021</v>
+        <v>1120</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>850</v>
+        <v>889</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>2033</v>
+        <v>2069</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1737</v>
+        <v>1647</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>4320</v>
+        <v>5230</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2488</v>
+        <v>2500</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2818</v>
+        <v>3091</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -1853,7 +1853,7 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1711</v>
+        <v>1735</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -1903,7 +1903,7 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1554</v>
+        <v>1577</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1953,7 +1953,7 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>78</v>
+        <v>145</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1196</v>
+        <v>1511</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1509</v>
+        <v>1964</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -2153,7 +2153,7 @@
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1234</v>
+        <v>2348</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -2203,7 +2203,7 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>371</v>
+        <v>498</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -2253,7 +2253,7 @@
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>527</v>
+        <v>1189</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2172</v>
+        <v>2155</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>2416</v>
+        <v>2578</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1327</v>
+        <v>1499</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2050</v>
+        <v>2129</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>5649</v>
+        <v>5879</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>5548</v>
+        <v>5594</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>5254</v>
+        <v>6042</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
@@ -2653,7 +2653,7 @@
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1512</v>
+        <v>1125</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
@@ -2703,7 +2703,7 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>2277</v>
+        <v>685</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>7253</v>
+        <v>6188</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
@@ -2803,7 +2803,7 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>17890</v>
+        <v>13947</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>9786</v>
+        <v>9830</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
@@ -2903,7 +2903,7 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>4394</v>
+        <v>4021</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
@@ -2953,7 +2953,7 @@
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>14712</v>
+        <v>19113</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
@@ -3114,7 +3114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M62"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6214,6 +6214,162 @@
         </is>
       </c>
       <c r="M62" s="22" t="inlineStr">
+        <is>
+          <t>APPROVED WITH PROTOCOL DEBT</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>Local-59</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 09:51:33</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>054419c</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
+        <is>
+          <t>intergration_testing</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>181803.272</v>
+      </c>
+      <c r="G63" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H63" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="I63" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J63" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>94.29%</t>
+        </is>
+      </c>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M63" s="19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>Local-60</t>
+        </is>
+      </c>
+      <c r="C64" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 10:06:09</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>054419c</t>
+        </is>
+      </c>
+      <c r="E64" s="10" t="inlineStr">
+        <is>
+          <t>intergration_testing</t>
+        </is>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>196220.965</v>
+      </c>
+      <c r="G64" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H64" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="I64" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="L64" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M64" s="22" t="inlineStr">
+        <is>
+          <t>APPROVED WITH PROTOCOL DEBT</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="10" t="inlineStr">
+        <is>
+          <t>Local-61</t>
+        </is>
+      </c>
+      <c r="C65" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 11:29:24</t>
+        </is>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
+        <is>
+          <t>054419c</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="inlineStr">
+        <is>
+          <t>intergration_testing</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>212101.148</v>
+      </c>
+      <c r="G65" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H65" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="I65" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="L65" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M65" s="22" t="inlineStr">
         <is>
           <t>APPROVED WITH PROTOCOL DEBT</t>
         </is>
@@ -6593,7 +6749,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>5203</v>
+        <v>3969</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -6603,7 +6759,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -6614,7 +6770,7 @@
       </c>
       <c r="C7" s="25" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>1.88%</t>
         </is>
       </c>
     </row>
@@ -6671,10 +6827,10 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>5136</v>
-      </c>
-      <c r="D13" s="16" t="n">
-        <v>1</v>
+        <v>3901</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0</v>
@@ -6690,10 +6846,10 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>0</v>
@@ -6791,7 +6947,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>10.00 Hz</t>
+          <t>4.00 Hz</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -6799,9 +6955,9 @@
           <t>5.0 Hz</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -6835,7 +6991,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>20.00 Hz</t>
+          <t>4.00 Hz</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -6866,7 +7022,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>333.9 ms</t>
+          <t>321.8 ms</t>
         </is>
       </c>
     </row>
@@ -6878,7 +7034,7 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>5.2 ms</t>
+          <t>3.1 ms</t>
         </is>
       </c>
     </row>
@@ -6890,7 +7046,7 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>4.4 ms</t>
+          <t>3.7 ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix MAVProxy streamrate telemetry frequency for GLOBAL_POSITION_INT and regenerate integration test reports
</commit_message>
<xml_diff>
--- a/test_frontend/reports/integration_test_report.xlsx
+++ b/test_frontend/reports/integration_test_report.xlsx
@@ -104,8 +104,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="006F42C1"/>
-        <bgColor rgb="006F42C1"/>
+        <fgColor rgb="0028A745"/>
+        <bgColor rgb="0028A745"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,14 +146,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0028A745"/>
-        <bgColor rgb="0028A745"/>
+        <fgColor rgb="00FD7E14"/>
+        <bgColor rgb="00FD7E14"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FD7E14"/>
-        <bgColor rgb="00FD7E14"/>
+        <fgColor rgb="006F42C1"/>
+        <bgColor rgb="006F42C1"/>
       </patternFill>
     </fill>
   </fills>
@@ -183,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -228,22 +228,19 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -619,7 +616,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="47" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
@@ -640,7 +637,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>RELEASE STATUS: APPROVED WITH PROTOCOL DEBT</t>
+          <t>RELEASE STATUS: APPROVED</t>
         </is>
       </c>
     </row>
@@ -685,7 +682,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>054419c</t>
+          <t>4f3508b</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -745,7 +742,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-19 11:29:24</t>
+          <t>2026-06-19 14:23:27</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -789,7 +786,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>03:32</t>
+          <t>03:20</t>
         </is>
       </c>
     </row>
@@ -858,7 +855,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>1.05 s</t>
+          <t>1.03 s</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -888,7 +885,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>4.82 s</t>
+          <t>4.74 s</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
@@ -918,7 +915,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>0.24 s</t>
+          <t>0.41 s</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1253,7 +1250,7 @@
         </is>
       </c>
       <c r="E3" s="6" t="n">
-        <v>454</v>
+        <v>156</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -1303,7 +1300,7 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>120</v>
+        <v>83</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1353,7 +1350,7 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>5891</v>
+        <v>6191</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1403,7 +1400,7 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>4950</v>
+        <v>4797</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -1453,7 +1450,7 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -1503,7 +1500,7 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>1120</v>
+        <v>1039</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -1553,7 +1550,7 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>889</v>
+        <v>882</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -1603,7 +1600,7 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>2069</v>
+        <v>2035</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -1653,7 +1650,7 @@
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>1647</v>
+        <v>1640</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
@@ -1703,7 +1700,7 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5230</v>
+        <v>4303</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -1753,7 +1750,7 @@
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>2500</v>
+        <v>2444</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
@@ -1803,7 +1800,7 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>3091</v>
+        <v>2813</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -1853,7 +1850,7 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1735</v>
+        <v>1710</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -1903,7 +1900,7 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1577</v>
+        <v>1556</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1953,7 +1950,7 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>145</v>
+        <v>56</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -2003,7 +2000,7 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1511</v>
+        <v>1004</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -2053,7 +2050,7 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -2103,7 +2100,7 @@
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>1964</v>
+        <v>1171</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -2153,7 +2150,7 @@
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>2348</v>
+        <v>1256</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -2203,7 +2200,7 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>498</v>
+        <v>309</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -2253,7 +2250,7 @@
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1189</v>
+        <v>775</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -2303,7 +2300,7 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>2155</v>
+        <v>2094</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -2353,7 +2350,7 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>2578</v>
+        <v>2353</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -2403,7 +2400,7 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1499</v>
+        <v>1128</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -2453,7 +2450,7 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2129</v>
+        <v>2029</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -2503,7 +2500,7 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>5879</v>
+        <v>4579</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -2553,7 +2550,7 @@
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>5594</v>
+        <v>5528</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
@@ -2603,7 +2600,7 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>6042</v>
+        <v>5253</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
@@ -2653,7 +2650,7 @@
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1125</v>
+        <v>822</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
@@ -2703,7 +2700,7 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>685</v>
+        <v>629</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -2753,7 +2750,7 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>6188</v>
+        <v>7602</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
@@ -2803,7 +2800,7 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>13947</v>
+        <v>12956</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -2853,7 +2850,7 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>9830</v>
+        <v>9766</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
@@ -2903,7 +2900,7 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>4021</v>
+        <v>6498</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
@@ -2953,7 +2950,7 @@
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>19113</v>
+        <v>14025</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
@@ -3114,7 +3111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6372,6 +6369,110 @@
       <c r="M65" s="22" t="inlineStr">
         <is>
           <t>APPROVED WITH PROTOCOL DEBT</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t>Local-62</t>
+        </is>
+      </c>
+      <c r="C66" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 11:54:42</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>4f3508b</t>
+        </is>
+      </c>
+      <c r="E66" s="10" t="inlineStr">
+        <is>
+          <t>intergration_testing</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>201458.55</v>
+      </c>
+      <c r="G66" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H66" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="I66" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J66" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>91.43%</t>
+        </is>
+      </c>
+      <c r="L66" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M66" s="19" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>Local-63</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>2026-06-19 14:23:27</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>4f3508b</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
+        <is>
+          <t>intergration_testing</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>200706.414</v>
+      </c>
+      <c r="G67" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="H67" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="I67" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="L67" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M67" s="20" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
         </is>
       </c>
     </row>
@@ -6749,7 +6850,7 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>3969</v>
+        <v>8282</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -6759,7 +6860,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -6768,9 +6869,9 @@
           <t>Overall Packet Loss Rate</t>
         </is>
       </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>1.88%</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>0.87%</t>
         </is>
       </c>
     </row>
@@ -6827,10 +6928,10 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>3901</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>0</v>
+        <v>8219</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>1</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0</v>
@@ -6846,16 +6947,16 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="26" t="n">
-        <v>3</v>
+      <c r="F14" s="25" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -6947,7 +7048,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>4.00 Hz</t>
+          <t>10.00 Hz</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -6955,9 +7056,9 @@
           <t>5.0 Hz</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -6969,7 +7070,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>4.00 Hz</t>
+          <t>10.00 Hz</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -6991,7 +7092,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>4.00 Hz</t>
+          <t>18.20 Hz</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -7022,7 +7123,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>321.8 ms</t>
+          <t>348.8 ms</t>
         </is>
       </c>
     </row>
@@ -7032,9 +7133,9 @@
           <t>Arm Command-ACK Latency</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
-        <is>
-          <t>3.1 ms</t>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>1.9 ms</t>
         </is>
       </c>
     </row>
@@ -7044,9 +7145,9 @@
           <t>Mode Switch Transition Latency</t>
         </is>
       </c>
-      <c r="C15" s="27" t="inlineStr">
-        <is>
-          <t>3.7 ms</t>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>7.3 ms</t>
         </is>
       </c>
     </row>

</xml_diff>